<commit_message>
Added two more shulkers with loot at tops of MInoc trees (climbing puzzle)
</commit_message>
<xml_diff>
--- a/spoilers/trades.xlsx
+++ b/spoilers/trades.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0296F742-0C33-46F1-A098-A3C0F3D704B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26527552-570C-4726-97D9-8BE2B99A3482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1266,7 +1266,7 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1725,7 +1725,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:L1048574"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1781,7 +1780,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
         <v>32</v>
       </c>
@@ -1815,7 +1814,7 @@
       </c>
       <c r="L2" s="36"/>
     </row>
-    <row r="3" spans="1:12" ht="52.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
         <v>32</v>
       </c>
@@ -1851,7 +1850,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="26.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>32</v>
       </c>
@@ -1887,7 +1886,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
         <v>32</v>
       </c>
@@ -1923,7 +1922,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
         <v>32</v>
       </c>
@@ -1959,7 +1958,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
         <v>32</v>
       </c>
@@ -1993,7 +1992,7 @@
       </c>
       <c r="L7" s="36"/>
     </row>
-    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
         <v>32</v>
       </c>
@@ -2027,7 +2026,7 @@
       </c>
       <c r="L8" s="36"/>
     </row>
-    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
         <v>32</v>
       </c>
@@ -2063,7 +2062,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="19" t="s">
         <v>32</v>
       </c>
@@ -2099,7 +2098,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:12" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="20" t="s">
         <v>32</v>
       </c>
@@ -2135,7 +2134,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
         <v>32</v>
       </c>
@@ -2169,7 +2168,7 @@
       </c>
       <c r="L12" s="36"/>
     </row>
-    <row r="13" spans="1:12" ht="79.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="79.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="19" t="s">
         <v>32</v>
       </c>
@@ -2207,7 +2206,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
         <v>32</v>
       </c>
@@ -2241,7 +2240,7 @@
       </c>
       <c r="L14" s="36"/>
     </row>
-    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="19" t="s">
         <v>32</v>
       </c>
@@ -2275,7 +2274,7 @@
       </c>
       <c r="L15" s="36"/>
     </row>
-    <row r="16" spans="1:12" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A16" s="19" t="s">
         <v>32</v>
       </c>
@@ -2311,7 +2310,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="19" t="s">
         <v>32</v>
       </c>
@@ -2347,7 +2346,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="39.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="19" t="s">
         <v>32</v>
       </c>
@@ -2385,7 +2384,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="19" t="s">
         <v>32</v>
       </c>
@@ -2419,7 +2418,7 @@
       </c>
       <c r="L19" s="36"/>
     </row>
-    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="19" t="s">
         <v>32</v>
       </c>
@@ -2453,7 +2452,7 @@
       </c>
       <c r="L20" s="36"/>
     </row>
-    <row r="21" spans="1:12" s="13" customFormat="1" ht="52.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" s="13" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A21" s="21" t="s">
         <v>32</v>
       </c>
@@ -2489,7 +2488,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="22" spans="1:12" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="21" t="s">
         <v>32</v>
       </c>
@@ -2523,7 +2522,7 @@
       </c>
       <c r="L22" s="38"/>
     </row>
-    <row r="23" spans="1:12" s="13" customFormat="1" ht="79.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" s="13" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A23" s="21" t="s">
         <v>32</v>
       </c>
@@ -2561,7 +2560,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:12" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="59" t="s">
         <v>32</v>
       </c>
@@ -2595,7 +2594,7 @@
       </c>
       <c r="L24" s="46"/>
     </row>
-    <row r="25" spans="1:12" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="59" t="s">
         <v>32</v>
       </c>
@@ -2629,7 +2628,7 @@
       </c>
       <c r="L25" s="46"/>
     </row>
-    <row r="26" spans="1:12" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="59" t="s">
         <v>32</v>
       </c>
@@ -2663,7 +2662,7 @@
       </c>
       <c r="L26" s="46"/>
     </row>
-    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="59" t="s">
         <v>32</v>
       </c>
@@ -2697,7 +2696,7 @@
       </c>
       <c r="L27" s="47"/>
     </row>
-    <row r="28" spans="1:12" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="59" t="s">
         <v>32</v>
       </c>
@@ -2733,7 +2732,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="29" spans="1:12" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="59" t="s">
         <v>32</v>
       </c>
@@ -2767,7 +2766,7 @@
       </c>
       <c r="L29" s="48"/>
     </row>
-    <row r="30" spans="1:12" s="8" customFormat="1" ht="112.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" s="8" customFormat="1" ht="112.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="59" t="s">
         <v>32</v>
       </c>
@@ -2805,7 +2804,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="31" spans="1:12" s="8" customFormat="1" ht="74.400000000000006" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" s="8" customFormat="1" ht="74.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="59" t="s">
         <v>32</v>
       </c>
@@ -2843,7 +2842,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A32" s="59" t="s">
         <v>32</v>
       </c>
@@ -2879,7 +2878,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A33" s="59" t="s">
         <v>32</v>
       </c>
@@ -2915,7 +2914,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A34" s="59" t="s">
         <v>32</v>
       </c>
@@ -2951,7 +2950,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="59" t="s">
         <v>32</v>
       </c>
@@ -2987,7 +2986,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="59" t="s">
         <v>32</v>
       </c>
@@ -3023,7 +3022,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="37" spans="1:12" s="30" customFormat="1" ht="88.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" s="30" customFormat="1" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="21" t="s">
         <v>32</v>
       </c>
@@ -3059,7 +3058,7 @@
       </c>
       <c r="L37" s="50"/>
     </row>
-    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="21" t="s">
         <v>32</v>
       </c>
@@ -3093,7 +3092,7 @@
       </c>
       <c r="L38" s="46"/>
     </row>
-    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="21" t="s">
         <v>32</v>
       </c>
@@ -3127,7 +3126,7 @@
       </c>
       <c r="L39" s="46"/>
     </row>
-    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" s="21" t="s">
         <v>32</v>
       </c>
@@ -3161,7 +3160,7 @@
       </c>
       <c r="L40" s="46"/>
     </row>
-    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" s="21" t="s">
         <v>32</v>
       </c>
@@ -3195,7 +3194,7 @@
       </c>
       <c r="L41" s="46"/>
     </row>
-    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" s="21" t="s">
         <v>32</v>
       </c>
@@ -3229,7 +3228,7 @@
       </c>
       <c r="L42" s="46"/>
     </row>
-    <row r="43" spans="1:12" ht="27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A43" s="59" t="s">
         <v>32</v>
       </c>
@@ -3265,7 +3264,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="44" spans="1:12" ht="13.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="59" t="s">
         <v>32</v>
       </c>
@@ -3301,7 +3300,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" s="59" t="s">
         <v>32</v>
       </c>
@@ -3337,7 +3336,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" s="59" t="s">
         <v>32</v>
       </c>
@@ -3373,7 +3372,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="59" t="s">
         <v>32</v>
       </c>
@@ -3407,7 +3406,7 @@
       </c>
       <c r="L47" s="46"/>
     </row>
-    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" s="59" t="s">
         <v>32</v>
       </c>
@@ -3441,7 +3440,7 @@
       </c>
       <c r="L48" s="46"/>
     </row>
-    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" s="59" t="s">
         <v>32</v>
       </c>
@@ -3475,7 +3474,7 @@
       </c>
       <c r="L49" s="46"/>
     </row>
-    <row r="50" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="59" t="s">
         <v>32</v>
       </c>
@@ -3509,7 +3508,7 @@
       </c>
       <c r="L50" s="46"/>
     </row>
-    <row r="51" spans="1:12" ht="40.200000000000003" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:12" ht="40.200000000000003" x14ac:dyDescent="0.3">
       <c r="A51" s="59" t="s">
         <v>32</v>
       </c>
@@ -3545,7 +3544,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="52" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" s="59" t="s">
         <v>32</v>
       </c>
@@ -3579,7 +3578,7 @@
       </c>
       <c r="L52" s="46"/>
     </row>
-    <row r="53" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53" s="59" t="s">
         <v>32</v>
       </c>
@@ -3613,7 +3612,7 @@
       </c>
       <c r="L53" s="46"/>
     </row>
-    <row r="54" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54" s="59" t="s">
         <v>32</v>
       </c>
@@ -3647,7 +3646,7 @@
       </c>
       <c r="L54" s="46"/>
     </row>
-    <row r="55" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A55" s="59" t="s">
         <v>32</v>
       </c>
@@ -3681,7 +3680,7 @@
       </c>
       <c r="L55" s="46"/>
     </row>
-    <row r="56" spans="1:12" ht="27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A56" s="59" t="s">
         <v>32</v>
       </c>
@@ -3717,7 +3716,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="57" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A57" s="59" t="s">
         <v>32</v>
       </c>
@@ -3753,7 +3752,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="58" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A58" s="59" t="s">
         <v>32</v>
       </c>
@@ -3789,7 +3788,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="59" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A59" s="59" t="s">
         <v>32</v>
       </c>
@@ -3823,7 +3822,7 @@
       </c>
       <c r="L59" s="48"/>
     </row>
-    <row r="60" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60" s="59" t="s">
         <v>32</v>
       </c>
@@ -3857,7 +3856,7 @@
       </c>
       <c r="L60" s="48"/>
     </row>
-    <row r="61" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A61" s="59" t="s">
         <v>32</v>
       </c>
@@ -3891,7 +3890,7 @@
       </c>
       <c r="L61" s="48"/>
     </row>
-    <row r="62" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A62" s="59" t="s">
         <v>32</v>
       </c>
@@ -3925,7 +3924,7 @@
       </c>
       <c r="L62" s="48"/>
     </row>
-    <row r="63" spans="1:12" s="27" customFormat="1" ht="25.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:12" s="27" customFormat="1" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="23" t="s">
         <v>32</v>
       </c>
@@ -3961,7 +3960,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="64" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A64" s="23" t="s">
         <v>32</v>
       </c>
@@ -3995,7 +3994,7 @@
       </c>
       <c r="L64" s="46"/>
     </row>
-    <row r="65" spans="1:12" s="27" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" s="23" t="s">
         <v>32</v>
       </c>
@@ -4031,7 +4030,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="66" spans="1:12" s="52" customFormat="1" ht="72.599999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:12" s="52" customFormat="1" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="33" t="s">
         <v>32</v>
       </c>
@@ -4067,7 +4066,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="67" spans="1:12" s="52" customFormat="1" ht="72.599999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:12" s="52" customFormat="1" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="33" t="s">
         <v>32</v>
       </c>
@@ -4105,7 +4104,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="68" spans="1:12" s="52" customFormat="1" ht="72.599999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:12" s="52" customFormat="1" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="23" t="s">
         <v>32</v>
       </c>
@@ -4141,7 +4140,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="69" spans="1:12" s="52" customFormat="1" ht="72.599999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:12" s="52" customFormat="1" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="23" t="s">
         <v>32</v>
       </c>
@@ -4177,7 +4176,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="70" spans="1:12" s="27" customFormat="1" ht="40.200000000000003" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:12" s="27" customFormat="1" ht="40.200000000000003" x14ac:dyDescent="0.3">
       <c r="A70" s="23" t="s">
         <v>32</v>
       </c>
@@ -4213,7 +4212,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="71" spans="1:12" s="27" customFormat="1" ht="40.200000000000003" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:12" s="27" customFormat="1" ht="40.200000000000003" x14ac:dyDescent="0.3">
       <c r="A71" s="23" t="s">
         <v>32</v>
       </c>
@@ -4249,7 +4248,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="72" spans="1:12" ht="40.200000000000003" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:12" ht="40.200000000000003" x14ac:dyDescent="0.3">
       <c r="A72" s="23" t="s">
         <v>32</v>
       </c>
@@ -4285,7 +4284,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A73" s="59" t="s">
         <v>149</v>
       </c>
@@ -4321,7 +4320,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A74" s="59" t="s">
         <v>149</v>
       </c>
@@ -4357,7 +4356,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A75" s="59" t="s">
         <v>149</v>
       </c>
@@ -4393,7 +4392,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A76" s="59" t="s">
         <v>149</v>
       </c>
@@ -4429,7 +4428,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="77" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A77" s="59" t="s">
         <v>149</v>
       </c>
@@ -4465,7 +4464,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="78" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A78" s="59" t="s">
         <v>149</v>
       </c>
@@ -4501,7 +4500,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="79" spans="1:12" ht="27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:12" ht="27" x14ac:dyDescent="0.3">
       <c r="A79" s="61" t="s">
         <v>164</v>
       </c>
@@ -4537,7 +4536,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A80" s="61" t="s">
         <v>164</v>
       </c>
@@ -4571,7 +4570,7 @@
       </c>
       <c r="L80" s="47"/>
     </row>
-    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A81" s="61" t="s">
         <v>164</v>
       </c>
@@ -4605,7 +4604,7 @@
       </c>
       <c r="L81" s="47"/>
     </row>
-    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A82" s="61" t="s">
         <v>164</v>
       </c>
@@ -4639,7 +4638,7 @@
       </c>
       <c r="L82" s="47"/>
     </row>
-    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A83" s="61" t="s">
         <v>164</v>
       </c>
@@ -4673,7 +4672,7 @@
       </c>
       <c r="L83" s="47"/>
     </row>
-    <row r="84" spans="1:12" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:12" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A84" s="26" t="s">
         <v>177</v>
       </c>
@@ -4709,7 +4708,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A85" s="26" t="s">
         <v>177</v>
       </c>
@@ -4743,7 +4742,7 @@
       </c>
       <c r="L85" s="56"/>
     </row>
-    <row r="86" spans="1:12" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:12" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A86" s="26" t="s">
         <v>177</v>
       </c>
@@ -4779,7 +4778,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="87" spans="1:12" s="27" customFormat="1" ht="276" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:12" s="27" customFormat="1" ht="276" x14ac:dyDescent="0.3">
       <c r="A87" s="28" t="s">
         <v>177</v>
       </c>
@@ -4817,7 +4816,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="88" spans="1:12" ht="53.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:12" ht="53.4" x14ac:dyDescent="0.3">
       <c r="A88" s="61" t="s">
         <v>177</v>
       </c>
@@ -4853,7 +4852,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="89" spans="1:12" ht="53.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:12" ht="53.4" x14ac:dyDescent="0.3">
       <c r="A89" s="61" t="s">
         <v>177</v>
       </c>
@@ -4889,7 +4888,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A90" s="61" t="s">
         <v>177</v>
       </c>
@@ -4923,7 +4922,7 @@
       </c>
       <c r="L90" s="56"/>
     </row>
-    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A91" s="61" t="s">
         <v>177</v>
       </c>
@@ -4957,7 +4956,7 @@
       </c>
       <c r="L91" s="47"/>
     </row>
-    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A92" s="61" t="s">
         <v>177</v>
       </c>
@@ -4991,7 +4990,7 @@
       </c>
       <c r="L92" s="47"/>
     </row>
-    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A93" s="61" t="s">
         <v>177</v>
       </c>
@@ -5025,7 +5024,7 @@
       </c>
       <c r="L93" s="47"/>
     </row>
-    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A94" s="63" t="s">
         <v>177</v>
       </c>
@@ -5043,7 +5042,7 @@
       <c r="K94" s="28"/>
       <c r="L94" s="47"/>
     </row>
-    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A95" s="66" t="s">
         <v>164</v>
       </c>
@@ -5061,7 +5060,7 @@
       <c r="K95" s="28"/>
       <c r="L95" s="47"/>
     </row>
-    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A96" s="66" t="s">
         <v>194</v>
       </c>
@@ -5079,7 +5078,7 @@
       <c r="K96" s="28"/>
       <c r="L96" s="47"/>
     </row>
-    <row r="97" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A97" s="66" t="s">
         <v>196</v>
       </c>
@@ -5097,7 +5096,7 @@
       <c r="K97" s="28"/>
       <c r="L97" s="47"/>
     </row>
-    <row r="98" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A98" s="67" t="s">
         <v>202</v>
       </c>
@@ -9151,13 +9150,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L145" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Minoc"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:L145" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="D51:D57 D2:D43 D59:D72 D114:D115 D117:D317 D74:D110" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"1,2,3,4,5"</formula1>

</xml_diff>